<commit_message>
Mehr Ausgaben in den Metriken: Zeiten, Parameter, Konfusionsmatrizen
</commit_message>
<xml_diff>
--- a/results/model_comparison_01.xlsx
+++ b/results/model_comparison_01.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -439,7 +439,10 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="215" customWidth="1" min="9" max="9"/>
+    <col width="216" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,6 +491,21 @@
           <t>Hyperparameters</t>
         </is>
       </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>vectorization_time_sec</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>training_time_sec</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>evaluation_time_sec</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -523,6 +541,15 @@
           <t>alpha: 1.0 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False | resampling: False</t>
         </is>
       </c>
+      <c r="J2" t="n">
+        <v>50.67616724967957</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.08211946487426749</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.1456139087677002</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -558,40 +585,58 @@
           <t>alpha: 1.0 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False | resampling: False</t>
         </is>
       </c>
+      <c r="J3" t="n">
+        <v>235.3060758113861</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.4123167991638183</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.7174978256225586</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SVM</t>
+          <t>Naive Bayes</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>run_01_50k</t>
+          <t>run_03_1250k</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.7217</v>
+        <v>0.7262446844118764</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5033466103993968</v>
+        <v>0.5436474110779915</v>
       </c>
       <c r="E4" t="n">
-        <v>0.422478356333673</v>
+        <v>0.3696821240817212</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4388695881248961</v>
+        <v>0.3912991253987072</v>
       </c>
       <c r="G4" t="n">
-        <v>160000</v>
+        <v>3561222</v>
       </c>
       <c r="H4" t="n">
-        <v>40000</v>
+        <v>890306</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>C: 1.0 | max_iter: 2000 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>alpha: 1.0 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False | resampling: False</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>379.5892918109894</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.8454170227050781</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1.320766925811768</v>
       </c>
     </row>
     <row r="5">
@@ -602,31 +647,40 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>run_02_250k</t>
+          <t>run_01_50k</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.741175</v>
+        <v>0.7217</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5413630317409346</v>
+        <v>0.5033466103993968</v>
       </c>
       <c r="E5" t="n">
-        <v>0.43378094950385</v>
+        <v>0.422478356333673</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4480824454682766</v>
+        <v>0.4388695881248961</v>
       </c>
       <c r="G5" t="n">
-        <v>800000</v>
+        <v>160000</v>
       </c>
       <c r="H5" t="n">
-        <v>200000</v>
+        <v>40000</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>C: 1.0 | max_iter: 2000 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 1.0 | max_iter: 2000 | class_weight: None | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>26.53803658485413</v>
+      </c>
+      <c r="K5" t="n">
+        <v>25.81752777099609</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.07040262222290029</v>
       </c>
     </row>
     <row r="6">
@@ -637,31 +691,40 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>run_04_1250k</t>
+          <t>run_02_250k</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.7537386022333894</v>
+        <v>0.741175</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5671098379771432</v>
+        <v>0.5413630317409346</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4351818972057671</v>
+        <v>0.43378094950385</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4494981216005155</v>
+        <v>0.4480824454682766</v>
       </c>
       <c r="G6" t="n">
-        <v>3561222</v>
+        <v>800000</v>
       </c>
       <c r="H6" t="n">
-        <v>890306</v>
+        <v>200000</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>C: 1.0 | max_iter: 2000 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 1.0 | max_iter: 2000 | class_weight: None | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>96.64133214950562</v>
+      </c>
+      <c r="K6" t="n">
+        <v>96.70594763755798</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.3011398315429687</v>
       </c>
     </row>
     <row r="7">
@@ -672,20 +735,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>run_05_1250k</t>
+          <t>run_03_1250k</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.7295637679629251</v>
+        <v>0.7537386022333894</v>
       </c>
       <c r="D7" t="n">
-        <v>0.501975320199012</v>
+        <v>0.5671098379771432</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5254035597942818</v>
+        <v>0.4351818972057671</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5090761975335786</v>
+        <v>0.4494981216005155</v>
       </c>
       <c r="G7" t="n">
         <v>3561222</v>
@@ -695,8 +758,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>C: 1.0 | max_iter: 2000 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 1.0 | max_iter: 2000 | class_weight: None | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>404.7021679878235</v>
+      </c>
+      <c r="K7" t="n">
+        <v>517.7515890598297</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1.423589944839478</v>
       </c>
     </row>
     <row r="8">
@@ -707,20 +779,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>run_06_1250k</t>
+          <t>run_04_1250k</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.7295873553587193</v>
+        <v>0.7536992899070657</v>
       </c>
       <c r="D8" t="n">
-        <v>0.5019759853811595</v>
+        <v>0.5672464165090474</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5253265458258006</v>
+        <v>0.4349332551580267</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5090426061576181</v>
+        <v>0.4491727372178027</v>
       </c>
       <c r="G8" t="n">
         <v>3561222</v>
@@ -730,43 +802,61 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>C: 0.5 | max_iter: 2000 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 0.5 | max_iter: 2000 | class_weight: None | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>372.7948234081268</v>
+      </c>
+      <c r="K8" t="n">
+        <v>561.1327376365662</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1.433217525482178</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Logistic Regression</t>
+          <t>SVM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>run_01_50k</t>
+          <t>run_05_1250k</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.727925</v>
+        <v>0.7295637679629251</v>
       </c>
       <c r="D9" t="n">
-        <v>0.5336110492786232</v>
+        <v>0.501975320199012</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4378957821097765</v>
+        <v>0.5254035597942818</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4608459534227099</v>
+        <v>0.5090761975335786</v>
       </c>
       <c r="G9" t="n">
-        <v>160000</v>
+        <v>3561222</v>
       </c>
       <c r="H9" t="n">
-        <v>40000</v>
+        <v>890306</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>C: 1.0 | max_iter: 1000 | solver: saga | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 1.0 | max_iter: 2000 | class_weight: balanced | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>395.7849805355072</v>
+      </c>
+      <c r="K9" t="n">
+        <v>586.5237317085266</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1.412526607513428</v>
       </c>
     </row>
     <row r="10">
@@ -777,31 +867,40 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>run_02_250k</t>
+          <t>run_01_50k</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.74392</v>
+        <v>0.727925</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5418137612226241</v>
+        <v>0.5336110492786232</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4596041157373801</v>
+        <v>0.4378957821097765</v>
       </c>
       <c r="F10" t="n">
-        <v>0.478312888651172</v>
+        <v>0.4608459534227099</v>
       </c>
       <c r="G10" t="n">
-        <v>800000</v>
+        <v>160000</v>
       </c>
       <c r="H10" t="n">
-        <v>200000</v>
+        <v>40000</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>C: 1.0 | max_iter: 1000 | solver: saga | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 1 | max_iter: 1000 | solver: saga | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>28.48625016212464</v>
+      </c>
+      <c r="K10" t="n">
+        <v>5.495212554931641</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.0660116672515869</v>
       </c>
     </row>
     <row r="11">
@@ -812,31 +911,40 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>run_04_1250k</t>
+          <t>run_02_250k</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.7581224882231502</v>
+        <v>0.74392</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5601319210697214</v>
+        <v>0.5418137612226241</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4686095040532082</v>
+        <v>0.4596041157373801</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4867652124873587</v>
+        <v>0.478312888651172</v>
       </c>
       <c r="G11" t="n">
-        <v>3561222</v>
+        <v>800000</v>
       </c>
       <c r="H11" t="n">
-        <v>890306</v>
+        <v>200000</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>C: 1.0 | max_iter: 1000 | solver: saga | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 1 | max_iter: 1000 | solver: saga | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>104.8704919815064</v>
+      </c>
+      <c r="K11" t="n">
+        <v>30.91805577278137</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.3123984336853027</v>
       </c>
     </row>
     <row r="12">
@@ -847,20 +955,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>run_05_1250k</t>
+          <t>run_03_1250k</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.7580270154306497</v>
+        <v>0.7581224882231502</v>
       </c>
       <c r="D12" t="n">
-        <v>0.5618477205400926</v>
+        <v>0.5601319210697214</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4667180766656752</v>
+        <v>0.4686095040532082</v>
       </c>
       <c r="F12" t="n">
-        <v>0.4852833677606842</v>
+        <v>0.4867652124873587</v>
       </c>
       <c r="G12" t="n">
         <v>3561222</v>
@@ -870,8 +978,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>C: 0.5 | max_iter: 1000 | solver: saga | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 1 | max_iter: 1000 | solver: saga | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>419.9295411109924</v>
+      </c>
+      <c r="K12" t="n">
+        <v>138.940390586853</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1.388064384460449</v>
       </c>
     </row>
     <row r="13">
@@ -882,20 +999,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>run_06_1250k</t>
+          <t>run_04_1250k</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.7577675540769129</v>
+        <v>0.7580270154306497</v>
       </c>
       <c r="D13" t="n">
-        <v>0.5628236813325947</v>
+        <v>0.5618477205400926</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4641787650417344</v>
+        <v>0.4667180766656752</v>
       </c>
       <c r="F13" t="n">
-        <v>0.483018885741485</v>
+        <v>0.4852833677606842</v>
       </c>
       <c r="G13" t="n">
         <v>3561222</v>
@@ -905,78 +1022,105 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>C: 0.5 | max_iter: 1000 | solver: lbfgs | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 0.5 | max_iter: 1000 | solver: saga | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>410.203469991684</v>
+      </c>
+      <c r="K13" t="n">
+        <v>137.4263887405396</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1.361344814300537</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Neural Network</t>
+          <t>Logistic Regression</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>run_01_50k</t>
+          <t>run_05_1250k</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.7323666666666667</v>
+        <v>0.7580270154306497</v>
       </c>
       <c r="D14" t="n">
-        <v>0.5366880659762961</v>
+        <v>0.5586133287025976</v>
       </c>
       <c r="E14" t="n">
-        <v>0.4359273450310343</v>
+        <v>0.4694856113214315</v>
       </c>
       <c r="F14" t="n">
-        <v>0.4497633295748368</v>
+        <v>0.4872803231174515</v>
       </c>
       <c r="G14" t="n">
-        <v>140000</v>
+        <v>3561222</v>
       </c>
       <c r="H14" t="n">
-        <v>30000</v>
+        <v>890306</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>hidden_units: 256 | dropout_rate: 0.3 | learning_rate: 0.001 | batch_size: 128 | epochs_trained: 4 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 2.0 | max_iter: 1000 | solver: saga | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>410.6496934890747</v>
+      </c>
+      <c r="K14" t="n">
+        <v>135.1459999084473</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1.35302472114563</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Neural Network</t>
+          <t>Logistic Regression</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>run_02_250k</t>
+          <t>run_06_1250k</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.74932</v>
+        <v>0.757897846358443</v>
       </c>
       <c r="D15" t="n">
-        <v>0.5470748136742001</v>
+        <v>0.5603745591145282</v>
       </c>
       <c r="E15" t="n">
-        <v>0.4676009093552323</v>
+        <v>0.467909485888231</v>
       </c>
       <c r="F15" t="n">
-        <v>0.4795572818427628</v>
+        <v>0.4863243132526415</v>
       </c>
       <c r="G15" t="n">
-        <v>700000</v>
+        <v>3561222</v>
       </c>
       <c r="H15" t="n">
-        <v>150000</v>
+        <v>890306</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>hidden_units: 256 | dropout_rate: 0.3 | learning_rate: 0.001 | batch_size: 128 | epochs_trained: 5 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
-        </is>
+          <t>C: 1.0 | max_iter: 1000 | solver: lbfgs | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>411.3313031196594</v>
+      </c>
+      <c r="K15" t="n">
+        <v>328.4829251766205</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1.343034267425537</v>
       </c>
     </row>
     <row r="16">
@@ -987,31 +1131,216 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>run_01_50k</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.7309333333333333</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.5139543429575986</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.4434634350181002</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.4352020965032038</v>
+      </c>
+      <c r="G16" t="n">
+        <v>140000</v>
+      </c>
+      <c r="H16" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>hidden_units: 256 | dropout_rate: 0.3 | learning_rate: 0.001 | batch_size: 128 | epochs_trained: 4 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>24.38829159736633</v>
+      </c>
+      <c r="K16" t="n">
+        <v>71.87666988372803</v>
+      </c>
+      <c r="L16" t="n">
+        <v>3.245606422424316</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Neural Network</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>run_02_250k</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.74848</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.5416273081199992</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.4667677590601342</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.4779364562261248</v>
+      </c>
+      <c r="G17" t="n">
+        <v>700000</v>
+      </c>
+      <c r="H17" t="n">
+        <v>150000</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>hidden_units: 256 | dropout_rate: 0.3 | learning_rate: 0.001 | batch_size: 128 | epochs_trained: 5 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>91.29603171348572</v>
+      </c>
+      <c r="K17" t="n">
+        <v>396.6433248519897</v>
+      </c>
+      <c r="L17" t="n">
+        <v>12.34358668327332</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Neural Network</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>run_03_1250k</t>
         </is>
       </c>
-      <c r="C16" t="n">
-        <v>0.765933835532326</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0.5623270173870718</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0.4826328934903353</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0.4983291544648182</v>
-      </c>
-      <c r="G16" t="n">
+      <c r="C18" t="n">
+        <v>0.7665628322825094</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.5671607175144933</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.4765052009583764</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.4853961210991128</v>
+      </c>
+      <c r="G18" t="n">
         <v>3116069</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H18" t="n">
         <v>667730</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>hidden_units: 256 | dropout_rate: 0.3 | learning_rate: 0.001 | batch_size: 128 | epochs_trained: 5 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
         </is>
+      </c>
+      <c r="J18" t="n">
+        <v>657.901956319809</v>
+      </c>
+      <c r="K18" t="n">
+        <v>2632.369967222214</v>
+      </c>
+      <c r="L18" t="n">
+        <v>69.28791046142578</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Neural Network</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>run_04_1250k</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.766997139562398</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.5654200237967045</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.4805771173152394</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.4976614535840012</v>
+      </c>
+      <c r="G19" t="n">
+        <v>3116069</v>
+      </c>
+      <c r="H19" t="n">
+        <v>667730</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>hidden_units: 256 | dropout_rate: 0.3 | learning_rate: 0.0005 | batch_size: 128 | epochs_trained: 5 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>367.4033930301666</v>
+      </c>
+      <c r="K19" t="n">
+        <v>2019.489515542984</v>
+      </c>
+      <c r="L19" t="n">
+        <v>61.34028339385986</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Neural Network</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>run_05_1250k</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.7673940065595375</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.5670491527231531</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.4844127795763525</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.5023712234363439</v>
+      </c>
+      <c r="G20" t="n">
+        <v>3116069</v>
+      </c>
+      <c r="H20" t="n">
+        <v>667730</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>hidden_units: 512 | dropout_rate: 0.3 | learning_rate: 0.0005 | batch_size: 128 | epochs_trained: 5 | max_features: 10000 | min_df: 2 | max_df: 0.95 | ngram_range: (1, 2) | stop_words: english | sublinear_tf: False</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>359.484735250473</v>
+      </c>
+      <c r="K20" t="n">
+        <v>3541.388725280762</v>
+      </c>
+      <c r="L20" t="n">
+        <v>90.3842840194702</v>
       </c>
     </row>
   </sheetData>

</xml_diff>